<commit_message>
revert to stable navette version V26
</commit_message>
<xml_diff>
--- a/navette_paie_template.xlsx
+++ b/navette_paie_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Younes\Desktop\RimH\service-charge-backend\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Younes\Desktop\RimH\service-charge-backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37AAE4BC-0F28-40FE-95F1-3C582B509E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E160B999-4A05-4AF1-A7BF-8FFCAB9CF4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3EC3FD9A-0BFA-4D4C-A65E-92466D302C16}"/>
   </bookViews>
@@ -96,9 +96,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="00000"/>
+    <numFmt numFmtId="166" formatCode="d/m/yy;@"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -351,7 +352,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -400,18 +401,30 @@
     <xf numFmtId="165" fontId="4" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -427,17 +440,11 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -756,7 +763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36609678-9012-4DAE-9960-D4AA0DD66C6F}">
-  <dimension ref="A1:T50"/>
+  <dimension ref="A1:T64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="40.5703125" customWidth="1"/>
@@ -767,10 +774,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
+      <c r="B1" s="26"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -791,8 +798,8 @@
       <c r="T1" s="1"/>
     </row>
     <row r="2" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23"/>
-      <c r="B2" s="24"/>
+      <c r="A2" s="27"/>
+      <c r="B2" s="28"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -813,50 +820,50 @@
       <c r="T2" s="1"/>
     </row>
     <row r="3" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="28" t="s">
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="27"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="28" t="s">
+      <c r="G3" s="20"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="27"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="28" t="s">
+      <c r="J3" s="20"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="27"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="28" t="s">
+      <c r="M3" s="20"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="P3" s="27"/>
-      <c r="Q3" s="29"/>
-      <c r="R3" s="20" t="s">
+      <c r="P3" s="20"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="S3" s="18" t="s">
+      <c r="S3" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="20" t="s">
+      <c r="T3" s="22" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="26"/>
-      <c r="B4" s="26"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
       <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
@@ -902,28 +909,28 @@
       <c r="Q4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="R4" s="21"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="21"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="25"/>
+      <c r="T4" s="23"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="17"/>
-      <c r="P5" s="17"/>
-      <c r="Q5" s="17"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="31"/>
       <c r="R5" s="17"/>
       <c r="S5" s="17"/>
       <c r="T5" s="17"/>
@@ -931,21 +938,21 @@
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="17"/>
       <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="17"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="31"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="31"/>
+      <c r="Q6" s="31"/>
       <c r="R6" s="17"/>
       <c r="S6" s="17"/>
       <c r="T6" s="17"/>
@@ -953,21 +960,21 @@
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="17"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="31"/>
+      <c r="K7" s="31"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="31"/>
+      <c r="N7" s="31"/>
+      <c r="O7" s="32"/>
+      <c r="P7" s="31"/>
+      <c r="Q7" s="31"/>
       <c r="R7" s="17"/>
       <c r="S7" s="17"/>
       <c r="T7" s="17"/>
@@ -975,21 +982,21 @@
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="17"/>
-      <c r="P8" s="17"/>
-      <c r="Q8" s="17"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="31"/>
+      <c r="L8" s="32"/>
+      <c r="M8" s="31"/>
+      <c r="N8" s="31"/>
+      <c r="O8" s="32"/>
+      <c r="P8" s="31"/>
+      <c r="Q8" s="31"/>
       <c r="R8" s="17"/>
       <c r="S8" s="17"/>
       <c r="T8" s="17"/>
@@ -997,21 +1004,21 @@
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="17"/>
-      <c r="P9" s="17"/>
-      <c r="Q9" s="17"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="32"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="31"/>
       <c r="R9" s="17"/>
       <c r="S9" s="17"/>
       <c r="T9" s="17"/>
@@ -1019,21 +1026,21 @@
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17"/>
-      <c r="O10" s="17"/>
-      <c r="P10" s="17"/>
-      <c r="Q10" s="17"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="32"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
+      <c r="O10" s="32"/>
+      <c r="P10" s="31"/>
+      <c r="Q10" s="31"/>
       <c r="R10" s="17"/>
       <c r="S10" s="17"/>
       <c r="T10" s="17"/>
@@ -1041,21 +1048,21 @@
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
-      <c r="O11" s="17"/>
-      <c r="P11" s="17"/>
-      <c r="Q11" s="17"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="32"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="31"/>
+      <c r="O11" s="32"/>
+      <c r="P11" s="31"/>
+      <c r="Q11" s="31"/>
       <c r="R11" s="17"/>
       <c r="S11" s="17"/>
       <c r="T11" s="17"/>
@@ -1063,21 +1070,21 @@
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="17"/>
-      <c r="O12" s="17"/>
-      <c r="P12" s="17"/>
-      <c r="Q12" s="17"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="32"/>
+      <c r="M12" s="31"/>
+      <c r="N12" s="31"/>
+      <c r="O12" s="32"/>
+      <c r="P12" s="31"/>
+      <c r="Q12" s="31"/>
       <c r="R12" s="17"/>
       <c r="S12" s="17"/>
       <c r="T12" s="17"/>
@@ -1085,21 +1092,21 @@
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="17"/>
       <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="17"/>
-      <c r="M13" s="17"/>
-      <c r="N13" s="17"/>
-      <c r="O13" s="17"/>
-      <c r="P13" s="17"/>
-      <c r="Q13" s="17"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="32"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="31"/>
+      <c r="O13" s="32"/>
+      <c r="P13" s="31"/>
+      <c r="Q13" s="31"/>
       <c r="R13" s="17"/>
       <c r="S13" s="17"/>
       <c r="T13" s="17"/>
@@ -1107,21 +1114,21 @@
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="17"/>
       <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
-      <c r="O14" s="17"/>
-      <c r="P14" s="17"/>
-      <c r="Q14" s="17"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="32"/>
+      <c r="M14" s="31"/>
+      <c r="N14" s="31"/>
+      <c r="O14" s="32"/>
+      <c r="P14" s="31"/>
+      <c r="Q14" s="31"/>
       <c r="R14" s="17"/>
       <c r="S14" s="17"/>
       <c r="T14" s="17"/>
@@ -1129,21 +1136,21 @@
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="17"/>
       <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="17"/>
-      <c r="M15" s="17"/>
-      <c r="N15" s="17"/>
-      <c r="O15" s="17"/>
-      <c r="P15" s="17"/>
-      <c r="Q15" s="17"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="32"/>
+      <c r="M15" s="31"/>
+      <c r="N15" s="31"/>
+      <c r="O15" s="32"/>
+      <c r="P15" s="31"/>
+      <c r="Q15" s="31"/>
       <c r="R15" s="17"/>
       <c r="S15" s="17"/>
       <c r="T15" s="17"/>
@@ -1151,21 +1158,21 @@
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="17"/>
       <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="17"/>
-      <c r="L16" s="17"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="17"/>
-      <c r="O16" s="17"/>
-      <c r="P16" s="17"/>
-      <c r="Q16" s="17"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="32"/>
+      <c r="M16" s="31"/>
+      <c r="N16" s="31"/>
+      <c r="O16" s="32"/>
+      <c r="P16" s="31"/>
+      <c r="Q16" s="31"/>
       <c r="R16" s="17"/>
       <c r="S16" s="17"/>
       <c r="T16" s="17"/>
@@ -1173,21 +1180,21 @@
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="17"/>
       <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="17"/>
-      <c r="Q17" s="17"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="31"/>
+      <c r="L17" s="32"/>
+      <c r="M17" s="31"/>
+      <c r="N17" s="31"/>
+      <c r="O17" s="32"/>
+      <c r="P17" s="31"/>
+      <c r="Q17" s="31"/>
       <c r="R17" s="17"/>
       <c r="S17" s="17"/>
       <c r="T17" s="17"/>
@@ -1195,21 +1202,21 @@
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="17"/>
       <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="17"/>
-      <c r="P18" s="17"/>
-      <c r="Q18" s="17"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+      <c r="L18" s="32"/>
+      <c r="M18" s="31"/>
+      <c r="N18" s="31"/>
+      <c r="O18" s="32"/>
+      <c r="P18" s="31"/>
+      <c r="Q18" s="31"/>
       <c r="R18" s="17"/>
       <c r="S18" s="17"/>
       <c r="T18" s="17"/>
@@ -1217,21 +1224,21 @@
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="17"/>
       <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
-      <c r="O19" s="17"/>
-      <c r="P19" s="17"/>
-      <c r="Q19" s="17"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="32"/>
+      <c r="M19" s="31"/>
+      <c r="N19" s="31"/>
+      <c r="O19" s="32"/>
+      <c r="P19" s="31"/>
+      <c r="Q19" s="31"/>
       <c r="R19" s="17"/>
       <c r="S19" s="17"/>
       <c r="T19" s="17"/>
@@ -1239,21 +1246,21 @@
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="17"/>
       <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
-      <c r="P20" s="17"/>
-      <c r="Q20" s="17"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="31"/>
+      <c r="L20" s="32"/>
+      <c r="M20" s="31"/>
+      <c r="N20" s="31"/>
+      <c r="O20" s="32"/>
+      <c r="P20" s="31"/>
+      <c r="Q20" s="31"/>
       <c r="R20" s="17"/>
       <c r="S20" s="17"/>
       <c r="T20" s="17"/>
@@ -1261,21 +1268,21 @@
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="17"/>
       <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="17"/>
-      <c r="O21" s="17"/>
-      <c r="P21" s="17"/>
-      <c r="Q21" s="17"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="32"/>
+      <c r="M21" s="31"/>
+      <c r="N21" s="31"/>
+      <c r="O21" s="32"/>
+      <c r="P21" s="31"/>
+      <c r="Q21" s="31"/>
       <c r="R21" s="17"/>
       <c r="S21" s="17"/>
       <c r="T21" s="17"/>
@@ -1283,21 +1290,21 @@
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" s="17"/>
       <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="17"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="17"/>
-      <c r="O22" s="17"/>
-      <c r="P22" s="17"/>
-      <c r="Q22" s="17"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
+      <c r="L22" s="32"/>
+      <c r="M22" s="31"/>
+      <c r="N22" s="31"/>
+      <c r="O22" s="32"/>
+      <c r="P22" s="31"/>
+      <c r="Q22" s="31"/>
       <c r="R22" s="17"/>
       <c r="S22" s="17"/>
       <c r="T22" s="17"/>
@@ -1305,21 +1312,21 @@
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" s="17"/>
       <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="17"/>
-      <c r="O23" s="17"/>
-      <c r="P23" s="17"/>
-      <c r="Q23" s="17"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
+      <c r="L23" s="32"/>
+      <c r="M23" s="31"/>
+      <c r="N23" s="31"/>
+      <c r="O23" s="32"/>
+      <c r="P23" s="31"/>
+      <c r="Q23" s="31"/>
       <c r="R23" s="17"/>
       <c r="S23" s="17"/>
       <c r="T23" s="17"/>
@@ -1327,21 +1334,21 @@
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="17"/>
       <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="17"/>
-      <c r="K24" s="17"/>
-      <c r="L24" s="17"/>
-      <c r="M24" s="17"/>
-      <c r="N24" s="17"/>
-      <c r="O24" s="17"/>
-      <c r="P24" s="17"/>
-      <c r="Q24" s="17"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
+      <c r="L24" s="32"/>
+      <c r="M24" s="31"/>
+      <c r="N24" s="31"/>
+      <c r="O24" s="32"/>
+      <c r="P24" s="31"/>
+      <c r="Q24" s="31"/>
       <c r="R24" s="17"/>
       <c r="S24" s="17"/>
       <c r="T24" s="17"/>
@@ -1349,21 +1356,21 @@
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="17"/>
       <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="17"/>
-      <c r="M25" s="17"/>
-      <c r="N25" s="17"/>
-      <c r="O25" s="17"/>
-      <c r="P25" s="17"/>
-      <c r="Q25" s="17"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="31"/>
+      <c r="K25" s="31"/>
+      <c r="L25" s="32"/>
+      <c r="M25" s="31"/>
+      <c r="N25" s="31"/>
+      <c r="O25" s="32"/>
+      <c r="P25" s="31"/>
+      <c r="Q25" s="31"/>
       <c r="R25" s="17"/>
       <c r="S25" s="17"/>
       <c r="T25" s="17"/>
@@ -1371,21 +1378,21 @@
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="17"/>
       <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="17"/>
-      <c r="M26" s="17"/>
-      <c r="N26" s="17"/>
-      <c r="O26" s="17"/>
-      <c r="P26" s="17"/>
-      <c r="Q26" s="17"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="32"/>
+      <c r="M26" s="31"/>
+      <c r="N26" s="31"/>
+      <c r="O26" s="32"/>
+      <c r="P26" s="31"/>
+      <c r="Q26" s="31"/>
       <c r="R26" s="17"/>
       <c r="S26" s="17"/>
       <c r="T26" s="17"/>
@@ -1393,21 +1400,21 @@
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="17"/>
       <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="17"/>
-      <c r="L27" s="17"/>
-      <c r="M27" s="17"/>
-      <c r="N27" s="17"/>
-      <c r="O27" s="17"/>
-      <c r="P27" s="17"/>
-      <c r="Q27" s="17"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="31"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="31"/>
+      <c r="K27" s="31"/>
+      <c r="L27" s="32"/>
+      <c r="M27" s="31"/>
+      <c r="N27" s="31"/>
+      <c r="O27" s="32"/>
+      <c r="P27" s="31"/>
+      <c r="Q27" s="31"/>
       <c r="R27" s="17"/>
       <c r="S27" s="17"/>
       <c r="T27" s="17"/>
@@ -1415,21 +1422,21 @@
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="17"/>
       <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="17"/>
-      <c r="L28" s="17"/>
-      <c r="M28" s="17"/>
-      <c r="N28" s="17"/>
-      <c r="O28" s="17"/>
-      <c r="P28" s="17"/>
-      <c r="Q28" s="17"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
+      <c r="L28" s="32"/>
+      <c r="M28" s="31"/>
+      <c r="N28" s="31"/>
+      <c r="O28" s="32"/>
+      <c r="P28" s="31"/>
+      <c r="Q28" s="31"/>
       <c r="R28" s="17"/>
       <c r="S28" s="17"/>
       <c r="T28" s="17"/>
@@ -1437,21 +1444,21 @@
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="17"/>
       <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
-      <c r="L29" s="17"/>
-      <c r="M29" s="17"/>
-      <c r="N29" s="17"/>
-      <c r="O29" s="17"/>
-      <c r="P29" s="17"/>
-      <c r="Q29" s="17"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="31"/>
+      <c r="K29" s="31"/>
+      <c r="L29" s="32"/>
+      <c r="M29" s="31"/>
+      <c r="N29" s="31"/>
+      <c r="O29" s="32"/>
+      <c r="P29" s="31"/>
+      <c r="Q29" s="31"/>
       <c r="R29" s="17"/>
       <c r="S29" s="17"/>
       <c r="T29" s="17"/>
@@ -1459,21 +1466,21 @@
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" s="17"/>
       <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-      <c r="K30" s="17"/>
-      <c r="L30" s="17"/>
-      <c r="M30" s="17"/>
-      <c r="N30" s="17"/>
-      <c r="O30" s="17"/>
-      <c r="P30" s="17"/>
-      <c r="Q30" s="17"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="31"/>
+      <c r="K30" s="31"/>
+      <c r="L30" s="32"/>
+      <c r="M30" s="31"/>
+      <c r="N30" s="31"/>
+      <c r="O30" s="32"/>
+      <c r="P30" s="31"/>
+      <c r="Q30" s="31"/>
       <c r="R30" s="17"/>
       <c r="S30" s="17"/>
       <c r="T30" s="17"/>
@@ -1481,21 +1488,21 @@
     <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" s="17"/>
       <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
-      <c r="L31" s="17"/>
-      <c r="M31" s="17"/>
-      <c r="N31" s="17"/>
-      <c r="O31" s="17"/>
-      <c r="P31" s="17"/>
-      <c r="Q31" s="17"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="31"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="31"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="31"/>
+      <c r="K31" s="31"/>
+      <c r="L31" s="32"/>
+      <c r="M31" s="31"/>
+      <c r="N31" s="31"/>
+      <c r="O31" s="32"/>
+      <c r="P31" s="31"/>
+      <c r="Q31" s="31"/>
       <c r="R31" s="17"/>
       <c r="S31" s="17"/>
       <c r="T31" s="17"/>
@@ -1503,21 +1510,21 @@
     <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" s="17"/>
       <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="17"/>
-      <c r="K32" s="17"/>
-      <c r="L32" s="17"/>
-      <c r="M32" s="17"/>
-      <c r="N32" s="17"/>
-      <c r="O32" s="17"/>
-      <c r="P32" s="17"/>
-      <c r="Q32" s="17"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="31"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="31"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="31"/>
+      <c r="K32" s="31"/>
+      <c r="L32" s="32"/>
+      <c r="M32" s="31"/>
+      <c r="N32" s="31"/>
+      <c r="O32" s="32"/>
+      <c r="P32" s="31"/>
+      <c r="Q32" s="31"/>
       <c r="R32" s="17"/>
       <c r="S32" s="17"/>
       <c r="T32" s="17"/>
@@ -1525,21 +1532,21 @@
     <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" s="17"/>
       <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="17"/>
-      <c r="M33" s="17"/>
-      <c r="N33" s="17"/>
-      <c r="O33" s="17"/>
-      <c r="P33" s="17"/>
-      <c r="Q33" s="17"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="31"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="31"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31"/>
+      <c r="L33" s="32"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="31"/>
+      <c r="O33" s="32"/>
+      <c r="P33" s="31"/>
+      <c r="Q33" s="31"/>
       <c r="R33" s="17"/>
       <c r="S33" s="17"/>
       <c r="T33" s="17"/>
@@ -1547,21 +1554,21 @@
     <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" s="17"/>
       <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="17"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="17"/>
-      <c r="K34" s="17"/>
-      <c r="L34" s="17"/>
-      <c r="M34" s="17"/>
-      <c r="N34" s="17"/>
-      <c r="O34" s="17"/>
-      <c r="P34" s="17"/>
-      <c r="Q34" s="17"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="31"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="32"/>
+      <c r="M34" s="31"/>
+      <c r="N34" s="31"/>
+      <c r="O34" s="32"/>
+      <c r="P34" s="31"/>
+      <c r="Q34" s="31"/>
       <c r="R34" s="17"/>
       <c r="S34" s="17"/>
       <c r="T34" s="17"/>
@@ -1569,21 +1576,21 @@
     <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" s="17"/>
       <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="17"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="17"/>
-      <c r="K35" s="17"/>
-      <c r="L35" s="17"/>
-      <c r="M35" s="17"/>
-      <c r="N35" s="17"/>
-      <c r="O35" s="17"/>
-      <c r="P35" s="17"/>
-      <c r="Q35" s="17"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="31"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="31"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="32"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="31"/>
+      <c r="L35" s="32"/>
+      <c r="M35" s="31"/>
+      <c r="N35" s="31"/>
+      <c r="O35" s="32"/>
+      <c r="P35" s="31"/>
+      <c r="Q35" s="31"/>
       <c r="R35" s="17"/>
       <c r="S35" s="17"/>
       <c r="T35" s="17"/>
@@ -1591,21 +1598,21 @@
     <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" s="17"/>
       <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
-      <c r="G36" s="17"/>
-      <c r="H36" s="17"/>
-      <c r="I36" s="17"/>
-      <c r="J36" s="17"/>
-      <c r="K36" s="17"/>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-      <c r="N36" s="17"/>
-      <c r="O36" s="17"/>
-      <c r="P36" s="17"/>
-      <c r="Q36" s="17"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="31"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="31"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="31"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="31"/>
+      <c r="O36" s="32"/>
+      <c r="P36" s="31"/>
+      <c r="Q36" s="31"/>
       <c r="R36" s="17"/>
       <c r="S36" s="17"/>
       <c r="T36" s="17"/>
@@ -1613,21 +1620,21 @@
     <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" s="17"/>
       <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
-      <c r="G37" s="17"/>
-      <c r="H37" s="17"/>
-      <c r="I37" s="17"/>
-      <c r="J37" s="17"/>
-      <c r="K37" s="17"/>
-      <c r="L37" s="17"/>
-      <c r="M37" s="17"/>
-      <c r="N37" s="17"/>
-      <c r="O37" s="17"/>
-      <c r="P37" s="17"/>
-      <c r="Q37" s="17"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="31"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="31"/>
+      <c r="H37" s="31"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="31"/>
+      <c r="K37" s="31"/>
+      <c r="L37" s="32"/>
+      <c r="M37" s="31"/>
+      <c r="N37" s="31"/>
+      <c r="O37" s="32"/>
+      <c r="P37" s="31"/>
+      <c r="Q37" s="31"/>
       <c r="R37" s="17"/>
       <c r="S37" s="17"/>
       <c r="T37" s="17"/>
@@ -1635,21 +1642,21 @@
     <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" s="17"/>
       <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="17"/>
-      <c r="F38" s="17"/>
-      <c r="G38" s="17"/>
-      <c r="H38" s="17"/>
-      <c r="I38" s="17"/>
-      <c r="J38" s="17"/>
-      <c r="K38" s="17"/>
-      <c r="L38" s="17"/>
-      <c r="M38" s="17"/>
-      <c r="N38" s="17"/>
-      <c r="O38" s="17"/>
-      <c r="P38" s="17"/>
-      <c r="Q38" s="17"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="31"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="31"/>
+      <c r="H38" s="31"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="31"/>
+      <c r="K38" s="31"/>
+      <c r="L38" s="32"/>
+      <c r="M38" s="31"/>
+      <c r="N38" s="31"/>
+      <c r="O38" s="32"/>
+      <c r="P38" s="31"/>
+      <c r="Q38" s="31"/>
       <c r="R38" s="17"/>
       <c r="S38" s="17"/>
       <c r="T38" s="17"/>
@@ -1657,21 +1664,21 @@
     <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" s="17"/>
       <c r="B39" s="17"/>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="17"/>
-      <c r="F39" s="17"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="17"/>
-      <c r="I39" s="17"/>
-      <c r="J39" s="17"/>
-      <c r="K39" s="17"/>
-      <c r="L39" s="17"/>
-      <c r="M39" s="17"/>
-      <c r="N39" s="17"/>
-      <c r="O39" s="17"/>
-      <c r="P39" s="17"/>
-      <c r="Q39" s="17"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="31"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="31"/>
+      <c r="H39" s="31"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="31"/>
+      <c r="K39" s="31"/>
+      <c r="L39" s="32"/>
+      <c r="M39" s="31"/>
+      <c r="N39" s="31"/>
+      <c r="O39" s="32"/>
+      <c r="P39" s="31"/>
+      <c r="Q39" s="31"/>
       <c r="R39" s="17"/>
       <c r="S39" s="17"/>
       <c r="T39" s="17"/>
@@ -1679,21 +1686,21 @@
     <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" s="17"/>
       <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="17"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
-      <c r="L40" s="17"/>
-      <c r="M40" s="17"/>
-      <c r="N40" s="17"/>
-      <c r="O40" s="17"/>
-      <c r="P40" s="17"/>
-      <c r="Q40" s="17"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="31"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="31"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="31"/>
+      <c r="K40" s="31"/>
+      <c r="L40" s="32"/>
+      <c r="M40" s="31"/>
+      <c r="N40" s="31"/>
+      <c r="O40" s="32"/>
+      <c r="P40" s="31"/>
+      <c r="Q40" s="31"/>
       <c r="R40" s="17"/>
       <c r="S40" s="17"/>
       <c r="T40" s="17"/>
@@ -1701,21 +1708,21 @@
     <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" s="17"/>
       <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="17"/>
-      <c r="I41" s="17"/>
-      <c r="J41" s="17"/>
-      <c r="K41" s="17"/>
-      <c r="L41" s="17"/>
-      <c r="M41" s="17"/>
-      <c r="N41" s="17"/>
-      <c r="O41" s="17"/>
-      <c r="P41" s="17"/>
-      <c r="Q41" s="17"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="31"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="31"/>
+      <c r="H41" s="31"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="31"/>
+      <c r="K41" s="31"/>
+      <c r="L41" s="32"/>
+      <c r="M41" s="31"/>
+      <c r="N41" s="31"/>
+      <c r="O41" s="32"/>
+      <c r="P41" s="31"/>
+      <c r="Q41" s="31"/>
       <c r="R41" s="17"/>
       <c r="S41" s="17"/>
       <c r="T41" s="17"/>
@@ -1723,21 +1730,21 @@
     <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" s="17"/>
       <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="17"/>
-      <c r="F42" s="17"/>
-      <c r="G42" s="17"/>
-      <c r="H42" s="17"/>
-      <c r="I42" s="17"/>
-      <c r="J42" s="17"/>
-      <c r="K42" s="17"/>
-      <c r="L42" s="17"/>
-      <c r="M42" s="17"/>
-      <c r="N42" s="17"/>
-      <c r="O42" s="17"/>
-      <c r="P42" s="17"/>
-      <c r="Q42" s="17"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="31"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="32"/>
+      <c r="J42" s="31"/>
+      <c r="K42" s="31"/>
+      <c r="L42" s="32"/>
+      <c r="M42" s="31"/>
+      <c r="N42" s="31"/>
+      <c r="O42" s="32"/>
+      <c r="P42" s="31"/>
+      <c r="Q42" s="31"/>
       <c r="R42" s="17"/>
       <c r="S42" s="17"/>
       <c r="T42" s="17"/>
@@ -1745,21 +1752,21 @@
     <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" s="17"/>
       <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
-      <c r="D43" s="17"/>
-      <c r="E43" s="17"/>
-      <c r="F43" s="17"/>
-      <c r="G43" s="17"/>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-      <c r="N43" s="17"/>
-      <c r="O43" s="17"/>
-      <c r="P43" s="17"/>
-      <c r="Q43" s="17"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="31"/>
+      <c r="E43" s="31"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="31"/>
+      <c r="H43" s="31"/>
+      <c r="I43" s="32"/>
+      <c r="J43" s="31"/>
+      <c r="K43" s="31"/>
+      <c r="L43" s="32"/>
+      <c r="M43" s="31"/>
+      <c r="N43" s="31"/>
+      <c r="O43" s="32"/>
+      <c r="P43" s="31"/>
+      <c r="Q43" s="31"/>
       <c r="R43" s="17"/>
       <c r="S43" s="17"/>
       <c r="T43" s="17"/>
@@ -1767,21 +1774,21 @@
     <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" s="17"/>
       <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17"/>
-      <c r="J44" s="17"/>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
-      <c r="N44" s="17"/>
-      <c r="O44" s="17"/>
-      <c r="P44" s="17"/>
-      <c r="Q44" s="17"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="31"/>
+      <c r="E44" s="31"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="31"/>
+      <c r="H44" s="31"/>
+      <c r="I44" s="32"/>
+      <c r="J44" s="31"/>
+      <c r="K44" s="31"/>
+      <c r="L44" s="32"/>
+      <c r="M44" s="31"/>
+      <c r="N44" s="31"/>
+      <c r="O44" s="32"/>
+      <c r="P44" s="31"/>
+      <c r="Q44" s="31"/>
       <c r="R44" s="17"/>
       <c r="S44" s="17"/>
       <c r="T44" s="17"/>
@@ -1789,21 +1796,21 @@
     <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" s="17"/>
       <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="17"/>
-      <c r="O45" s="17"/>
-      <c r="P45" s="17"/>
-      <c r="Q45" s="17"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="31"/>
+      <c r="E45" s="31"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="31"/>
+      <c r="H45" s="31"/>
+      <c r="I45" s="32"/>
+      <c r="J45" s="31"/>
+      <c r="K45" s="31"/>
+      <c r="L45" s="32"/>
+      <c r="M45" s="31"/>
+      <c r="N45" s="31"/>
+      <c r="O45" s="32"/>
+      <c r="P45" s="31"/>
+      <c r="Q45" s="31"/>
       <c r="R45" s="17"/>
       <c r="S45" s="17"/>
       <c r="T45" s="17"/>
@@ -1811,21 +1818,21 @@
     <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" s="17"/>
       <c r="B46" s="17"/>
-      <c r="C46" s="17"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="17"/>
-      <c r="G46" s="17"/>
-      <c r="H46" s="17"/>
-      <c r="I46" s="17"/>
-      <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
-      <c r="L46" s="17"/>
-      <c r="M46" s="17"/>
-      <c r="N46" s="17"/>
-      <c r="O46" s="17"/>
-      <c r="P46" s="17"/>
-      <c r="Q46" s="17"/>
+      <c r="C46" s="32"/>
+      <c r="D46" s="31"/>
+      <c r="E46" s="31"/>
+      <c r="F46" s="32"/>
+      <c r="G46" s="31"/>
+      <c r="H46" s="31"/>
+      <c r="I46" s="32"/>
+      <c r="J46" s="31"/>
+      <c r="K46" s="31"/>
+      <c r="L46" s="32"/>
+      <c r="M46" s="31"/>
+      <c r="N46" s="31"/>
+      <c r="O46" s="32"/>
+      <c r="P46" s="31"/>
+      <c r="Q46" s="31"/>
       <c r="R46" s="17"/>
       <c r="S46" s="17"/>
       <c r="T46" s="17"/>
@@ -1833,124 +1840,427 @@
     <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" s="17"/>
       <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="17"/>
-      <c r="I47" s="17"/>
-      <c r="J47" s="17"/>
-      <c r="K47" s="17"/>
-      <c r="L47" s="17"/>
-      <c r="M47" s="17"/>
-      <c r="N47" s="17"/>
-      <c r="O47" s="17"/>
-      <c r="P47" s="17"/>
-      <c r="Q47" s="17"/>
+      <c r="C47" s="32"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="31"/>
+      <c r="F47" s="32"/>
+      <c r="G47" s="31"/>
+      <c r="H47" s="31"/>
+      <c r="I47" s="32"/>
+      <c r="J47" s="31"/>
+      <c r="K47" s="31"/>
+      <c r="L47" s="32"/>
+      <c r="M47" s="31"/>
+      <c r="N47" s="31"/>
+      <c r="O47" s="32"/>
+      <c r="P47" s="31"/>
+      <c r="Q47" s="31"/>
       <c r="R47" s="17"/>
       <c r="S47" s="17"/>
       <c r="T47" s="17"/>
     </row>
-    <row r="48" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A48" s="16"/>
-      <c r="B48" s="6"/>
-      <c r="C48" s="7">
-        <f>SUM(C5:C47)</f>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A48" s="17"/>
+      <c r="B48" s="17"/>
+      <c r="C48" s="32"/>
+      <c r="D48" s="31"/>
+      <c r="E48" s="31"/>
+      <c r="F48" s="32"/>
+      <c r="G48" s="31"/>
+      <c r="H48" s="31"/>
+      <c r="I48" s="32"/>
+      <c r="J48" s="31"/>
+      <c r="K48" s="31"/>
+      <c r="L48" s="32"/>
+      <c r="M48" s="31"/>
+      <c r="N48" s="31"/>
+      <c r="O48" s="32"/>
+      <c r="P48" s="31"/>
+      <c r="Q48" s="31"/>
+      <c r="R48" s="17"/>
+      <c r="S48" s="17"/>
+      <c r="T48" s="17"/>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A49" s="17"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="32"/>
+      <c r="D49" s="31"/>
+      <c r="E49" s="31"/>
+      <c r="F49" s="32"/>
+      <c r="G49" s="31"/>
+      <c r="H49" s="31"/>
+      <c r="I49" s="32"/>
+      <c r="J49" s="31"/>
+      <c r="K49" s="31"/>
+      <c r="L49" s="32"/>
+      <c r="M49" s="31"/>
+      <c r="N49" s="31"/>
+      <c r="O49" s="32"/>
+      <c r="P49" s="31"/>
+      <c r="Q49" s="31"/>
+      <c r="R49" s="17"/>
+      <c r="S49" s="17"/>
+      <c r="T49" s="17"/>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A50" s="17"/>
+      <c r="B50" s="17"/>
+      <c r="C50" s="32"/>
+      <c r="D50" s="31"/>
+      <c r="E50" s="31"/>
+      <c r="F50" s="32"/>
+      <c r="G50" s="31"/>
+      <c r="H50" s="31"/>
+      <c r="I50" s="32"/>
+      <c r="J50" s="31"/>
+      <c r="K50" s="31"/>
+      <c r="L50" s="32"/>
+      <c r="M50" s="31"/>
+      <c r="N50" s="31"/>
+      <c r="O50" s="32"/>
+      <c r="P50" s="31"/>
+      <c r="Q50" s="31"/>
+      <c r="R50" s="17"/>
+      <c r="S50" s="17"/>
+      <c r="T50" s="17"/>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A51" s="17"/>
+      <c r="B51" s="17"/>
+      <c r="C51" s="32"/>
+      <c r="D51" s="31"/>
+      <c r="E51" s="31"/>
+      <c r="F51" s="32"/>
+      <c r="G51" s="31"/>
+      <c r="H51" s="31"/>
+      <c r="I51" s="32"/>
+      <c r="J51" s="31"/>
+      <c r="K51" s="31"/>
+      <c r="L51" s="32"/>
+      <c r="M51" s="31"/>
+      <c r="N51" s="31"/>
+      <c r="O51" s="32"/>
+      <c r="P51" s="31"/>
+      <c r="Q51" s="31"/>
+      <c r="R51" s="17"/>
+      <c r="S51" s="17"/>
+      <c r="T51" s="17"/>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A52" s="17"/>
+      <c r="B52" s="17"/>
+      <c r="C52" s="32"/>
+      <c r="D52" s="31"/>
+      <c r="E52" s="31"/>
+      <c r="F52" s="32"/>
+      <c r="G52" s="31"/>
+      <c r="H52" s="31"/>
+      <c r="I52" s="32"/>
+      <c r="J52" s="31"/>
+      <c r="K52" s="31"/>
+      <c r="L52" s="32"/>
+      <c r="M52" s="31"/>
+      <c r="N52" s="31"/>
+      <c r="O52" s="32"/>
+      <c r="P52" s="31"/>
+      <c r="Q52" s="31"/>
+      <c r="R52" s="17"/>
+      <c r="S52" s="17"/>
+      <c r="T52" s="17"/>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A53" s="17"/>
+      <c r="B53" s="17"/>
+      <c r="C53" s="32"/>
+      <c r="D53" s="31"/>
+      <c r="E53" s="31"/>
+      <c r="F53" s="32"/>
+      <c r="G53" s="31"/>
+      <c r="H53" s="31"/>
+      <c r="I53" s="32"/>
+      <c r="J53" s="31"/>
+      <c r="K53" s="31"/>
+      <c r="L53" s="32"/>
+      <c r="M53" s="31"/>
+      <c r="N53" s="31"/>
+      <c r="O53" s="32"/>
+      <c r="P53" s="31"/>
+      <c r="Q53" s="31"/>
+      <c r="R53" s="17"/>
+      <c r="S53" s="17"/>
+      <c r="T53" s="17"/>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A54" s="17"/>
+      <c r="B54" s="17"/>
+      <c r="C54" s="32"/>
+      <c r="D54" s="31"/>
+      <c r="E54" s="31"/>
+      <c r="F54" s="32"/>
+      <c r="G54" s="31"/>
+      <c r="H54" s="31"/>
+      <c r="I54" s="32"/>
+      <c r="J54" s="31"/>
+      <c r="K54" s="31"/>
+      <c r="L54" s="32"/>
+      <c r="M54" s="31"/>
+      <c r="N54" s="31"/>
+      <c r="O54" s="32"/>
+      <c r="P54" s="31"/>
+      <c r="Q54" s="31"/>
+      <c r="R54" s="17"/>
+      <c r="S54" s="17"/>
+      <c r="T54" s="17"/>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A55" s="17"/>
+      <c r="B55" s="17"/>
+      <c r="C55" s="32"/>
+      <c r="D55" s="31"/>
+      <c r="E55" s="31"/>
+      <c r="F55" s="32"/>
+      <c r="G55" s="31"/>
+      <c r="H55" s="31"/>
+      <c r="I55" s="32"/>
+      <c r="J55" s="31"/>
+      <c r="K55" s="31"/>
+      <c r="L55" s="32"/>
+      <c r="M55" s="31"/>
+      <c r="N55" s="31"/>
+      <c r="O55" s="32"/>
+      <c r="P55" s="31"/>
+      <c r="Q55" s="31"/>
+      <c r="R55" s="17"/>
+      <c r="S55" s="17"/>
+      <c r="T55" s="17"/>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A56" s="17"/>
+      <c r="B56" s="17"/>
+      <c r="C56" s="32"/>
+      <c r="D56" s="31"/>
+      <c r="E56" s="31"/>
+      <c r="F56" s="32"/>
+      <c r="G56" s="31"/>
+      <c r="H56" s="31"/>
+      <c r="I56" s="32"/>
+      <c r="J56" s="31"/>
+      <c r="K56" s="31"/>
+      <c r="L56" s="32"/>
+      <c r="M56" s="31"/>
+      <c r="N56" s="31"/>
+      <c r="O56" s="32"/>
+      <c r="P56" s="31"/>
+      <c r="Q56" s="31"/>
+      <c r="R56" s="17"/>
+      <c r="S56" s="17"/>
+      <c r="T56" s="17"/>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A57" s="17"/>
+      <c r="B57" s="17"/>
+      <c r="C57" s="32"/>
+      <c r="D57" s="31"/>
+      <c r="E57" s="31"/>
+      <c r="F57" s="32"/>
+      <c r="G57" s="31"/>
+      <c r="H57" s="31"/>
+      <c r="I57" s="32"/>
+      <c r="J57" s="31"/>
+      <c r="K57" s="31"/>
+      <c r="L57" s="32"/>
+      <c r="M57" s="31"/>
+      <c r="N57" s="31"/>
+      <c r="O57" s="32"/>
+      <c r="P57" s="31"/>
+      <c r="Q57" s="31"/>
+      <c r="R57" s="17"/>
+      <c r="S57" s="17"/>
+      <c r="T57" s="17"/>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A58" s="17"/>
+      <c r="B58" s="17"/>
+      <c r="C58" s="32"/>
+      <c r="D58" s="31"/>
+      <c r="E58" s="31"/>
+      <c r="F58" s="32"/>
+      <c r="G58" s="31"/>
+      <c r="H58" s="31"/>
+      <c r="I58" s="32"/>
+      <c r="J58" s="31"/>
+      <c r="K58" s="31"/>
+      <c r="L58" s="32"/>
+      <c r="M58" s="31"/>
+      <c r="N58" s="31"/>
+      <c r="O58" s="32"/>
+      <c r="P58" s="31"/>
+      <c r="Q58" s="31"/>
+      <c r="R58" s="17"/>
+      <c r="S58" s="17"/>
+      <c r="T58" s="17"/>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A59" s="17"/>
+      <c r="B59" s="17"/>
+      <c r="C59" s="32"/>
+      <c r="D59" s="31"/>
+      <c r="E59" s="31"/>
+      <c r="F59" s="32"/>
+      <c r="G59" s="31"/>
+      <c r="H59" s="31"/>
+      <c r="I59" s="32"/>
+      <c r="J59" s="31"/>
+      <c r="K59" s="31"/>
+      <c r="L59" s="32"/>
+      <c r="M59" s="31"/>
+      <c r="N59" s="31"/>
+      <c r="O59" s="32"/>
+      <c r="P59" s="31"/>
+      <c r="Q59" s="31"/>
+      <c r="R59" s="17"/>
+      <c r="S59" s="17"/>
+      <c r="T59" s="17"/>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A60" s="17"/>
+      <c r="B60" s="17"/>
+      <c r="C60" s="32"/>
+      <c r="D60" s="31"/>
+      <c r="E60" s="31"/>
+      <c r="F60" s="32"/>
+      <c r="G60" s="31"/>
+      <c r="H60" s="31"/>
+      <c r="I60" s="32"/>
+      <c r="J60" s="31"/>
+      <c r="K60" s="31"/>
+      <c r="L60" s="32"/>
+      <c r="M60" s="31"/>
+      <c r="N60" s="31"/>
+      <c r="O60" s="32"/>
+      <c r="P60" s="31"/>
+      <c r="Q60" s="31"/>
+      <c r="R60" s="17"/>
+      <c r="S60" s="17"/>
+      <c r="T60" s="17"/>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A61" s="17"/>
+      <c r="B61" s="17"/>
+      <c r="C61" s="32"/>
+      <c r="D61" s="31"/>
+      <c r="E61" s="31"/>
+      <c r="F61" s="32"/>
+      <c r="G61" s="31"/>
+      <c r="H61" s="31"/>
+      <c r="I61" s="32"/>
+      <c r="J61" s="31"/>
+      <c r="K61" s="31"/>
+      <c r="L61" s="32"/>
+      <c r="M61" s="31"/>
+      <c r="N61" s="31"/>
+      <c r="O61" s="32"/>
+      <c r="P61" s="31"/>
+      <c r="Q61" s="31"/>
+      <c r="R61" s="17"/>
+      <c r="S61" s="17"/>
+      <c r="T61" s="17"/>
+    </row>
+    <row r="62" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A62" s="16"/>
+      <c r="B62" s="6"/>
+      <c r="C62" s="7">
+        <f>SUM(C5:C61)</f>
         <v>0</v>
       </c>
-      <c r="D48" s="7"/>
-      <c r="E48" s="7"/>
-      <c r="F48" s="7">
-        <f>SUM(F5:F47)</f>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7">
+        <f>SUM(F5:F61)</f>
         <v>0</v>
       </c>
-      <c r="G48" s="7"/>
-      <c r="H48" s="7"/>
-      <c r="I48" s="8">
-        <f>SUM(I4:I47)</f>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="8">
+        <f>SUM(I4:I61)</f>
         <v>0</v>
       </c>
-      <c r="J48" s="7"/>
-      <c r="K48" s="7"/>
-      <c r="L48" s="7">
-        <f>SUM(L5:L47)</f>
+      <c r="J62" s="7"/>
+      <c r="K62" s="7"/>
+      <c r="L62" s="7">
+        <f>SUM(L5:L61)</f>
         <v>0</v>
       </c>
-      <c r="M48" s="7"/>
-      <c r="N48" s="7"/>
-      <c r="O48" s="7">
+      <c r="M62" s="7"/>
+      <c r="N62" s="7"/>
+      <c r="O62" s="7">
         <v>0</v>
       </c>
-      <c r="P48" s="7"/>
-      <c r="Q48" s="7"/>
-      <c r="R48" s="9"/>
-      <c r="S48" s="10">
-        <f>SUM(S5:S47)</f>
+      <c r="P62" s="7"/>
+      <c r="Q62" s="7"/>
+      <c r="R62" s="9"/>
+      <c r="S62" s="10">
+        <f>SUM(S5:S61)</f>
         <v>0</v>
       </c>
-      <c r="T48" s="10">
-        <f>SUM(T5:T47)</f>
+      <c r="T62" s="10">
+        <f>SUM(T5:T61)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="7"/>
-      <c r="B49" s="11" t="s">
+    <row r="63" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A63" s="7"/>
+      <c r="B63" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C49" s="12"/>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="12"/>
-      <c r="G49" s="1"/>
-      <c r="H49" s="1"/>
-      <c r="I49" s="12"/>
-      <c r="J49" s="1"/>
-      <c r="K49" s="1"/>
-      <c r="L49" s="12"/>
-      <c r="M49" s="1"/>
-      <c r="N49" s="6"/>
-      <c r="O49" s="12"/>
-      <c r="P49" s="1"/>
-      <c r="Q49" s="1"/>
-      <c r="R49" s="1"/>
-      <c r="S49" s="13"/>
-      <c r="T49" s="13"/>
-    </row>
-    <row r="50" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A50" s="7"/>
-      <c r="B50" s="14" t="s">
+      <c r="C63" s="12"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="12"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+      <c r="I63" s="12"/>
+      <c r="J63" s="1"/>
+      <c r="K63" s="1"/>
+      <c r="L63" s="12"/>
+      <c r="M63" s="1"/>
+      <c r="N63" s="6"/>
+      <c r="O63" s="12"/>
+      <c r="P63" s="1"/>
+      <c r="Q63" s="1"/>
+      <c r="R63" s="1"/>
+      <c r="S63" s="13"/>
+      <c r="T63" s="13"/>
+    </row>
+    <row r="64" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A64" s="7"/>
+      <c r="B64" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C50" s="12"/>
-      <c r="D50" s="1"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="12"/>
-      <c r="G50" s="1"/>
-      <c r="H50" s="1"/>
-      <c r="I50" s="12"/>
-      <c r="J50" s="1"/>
-      <c r="K50" s="1"/>
-      <c r="L50" s="12"/>
-      <c r="M50" s="30" t="s">
+      <c r="C64" s="12"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="14"/>
+      <c r="F64" s="12"/>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+      <c r="I64" s="12"/>
+      <c r="J64" s="1"/>
+      <c r="K64" s="1"/>
+      <c r="L64" s="12"/>
+      <c r="M64" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="N50" s="30"/>
-      <c r="O50" s="30"/>
-      <c r="P50" s="30"/>
-      <c r="Q50" s="30"/>
-      <c r="R50" s="30"/>
-      <c r="S50" s="1"/>
-      <c r="T50" s="1"/>
+      <c r="N64" s="18"/>
+      <c r="O64" s="18"/>
+      <c r="P64" s="18"/>
+      <c r="Q64" s="18"/>
+      <c r="R64" s="18"/>
+      <c r="S64" s="1"/>
+      <c r="T64" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="M50:R50"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="L3:N3"/>
-    <mergeCell ref="O3:Q3"/>
-    <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
     <mergeCell ref="A1:B1"/>
@@ -1959,26 +2269,32 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:H3"/>
+    <mergeCell ref="M64:R64"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="L3:N3"/>
+    <mergeCell ref="O3:Q3"/>
+    <mergeCell ref="R3:R4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="dc189c0f-d569-423c-8bd8-1cb2ef291c21" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="dc189c0f-d569-423c-8bd8-1cb2ef291c21" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2176,6 +2492,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38AA6C2C-1214-4927-9979-113A2D4502E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52C24A3E-6A2C-40E5-B34D-1555475543C6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -2187,14 +2511,6 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38AA6C2C-1214-4927-9979-113A2D4502E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
revert to stable navette version V27
</commit_message>
<xml_diff>
--- a/navette_paie_template.xlsx
+++ b/navette_paie_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Younes\Desktop\RimH\service-charge-backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E160B999-4A05-4AF1-A7BF-8FFCAB9CF4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B51DDD30-A83D-4EB1-86D7-D0A61B946F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3EC3FD9A-0BFA-4D4C-A65E-92466D302C16}"/>
   </bookViews>
@@ -401,50 +401,50 @@
     <xf numFmtId="165" fontId="4" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -774,10 +774,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
+      <c r="B1" s="24"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -798,8 +798,8 @@
       <c r="T1" s="1"/>
     </row>
     <row r="2" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27"/>
-      <c r="B2" s="28"/>
+      <c r="A2" s="25"/>
+      <c r="B2" s="26"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -820,41 +820,41 @@
       <c r="T2" s="1"/>
     </row>
     <row r="3" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="19" t="s">
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="20"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="19" t="s">
+      <c r="G3" s="29"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="20"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="19" t="s">
+      <c r="J3" s="29"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="20"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="19" t="s">
+      <c r="M3" s="29"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="P3" s="20"/>
-      <c r="Q3" s="21"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="31"/>
       <c r="R3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="S3" s="24" t="s">
+      <c r="S3" s="20" t="s">
         <v>9</v>
       </c>
       <c r="T3" s="22" t="s">
@@ -862,8 +862,8 @@
       </c>
     </row>
     <row r="4" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="30"/>
-      <c r="B4" s="30"/>
+      <c r="A4" s="28"/>
+      <c r="B4" s="28"/>
       <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
@@ -910,27 +910,27 @@
         <v>14</v>
       </c>
       <c r="R4" s="23"/>
-      <c r="S4" s="25"/>
+      <c r="S4" s="21"/>
       <c r="T4" s="23"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="31"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="32"/>
-      <c r="M5" s="31"/>
-      <c r="N5" s="31"/>
-      <c r="O5" s="32"/>
-      <c r="P5" s="31"/>
-      <c r="Q5" s="31"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
       <c r="R5" s="17"/>
       <c r="S5" s="17"/>
       <c r="T5" s="17"/>
@@ -938,21 +938,21 @@
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="17"/>
       <c r="B6" s="17"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="31"/>
-      <c r="K6" s="31"/>
-      <c r="L6" s="32"/>
-      <c r="M6" s="31"/>
-      <c r="N6" s="31"/>
-      <c r="O6" s="32"/>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="31"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
       <c r="R6" s="17"/>
       <c r="S6" s="17"/>
       <c r="T6" s="17"/>
@@ -960,21 +960,21 @@
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="31"/>
-      <c r="L7" s="32"/>
-      <c r="M7" s="31"/>
-      <c r="N7" s="31"/>
-      <c r="O7" s="32"/>
-      <c r="P7" s="31"/>
-      <c r="Q7" s="31"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
       <c r="R7" s="17"/>
       <c r="S7" s="17"/>
       <c r="T7" s="17"/>
@@ -982,21 +982,21 @@
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="31"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="31"/>
-      <c r="N8" s="31"/>
-      <c r="O8" s="32"/>
-      <c r="P8" s="31"/>
-      <c r="Q8" s="31"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="18"/>
+      <c r="N8" s="18"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="18"/>
+      <c r="Q8" s="18"/>
       <c r="R8" s="17"/>
       <c r="S8" s="17"/>
       <c r="T8" s="17"/>
@@ -1004,21 +1004,21 @@
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
-      <c r="C9" s="32"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="32"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31"/>
-      <c r="L9" s="32"/>
-      <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="32"/>
-      <c r="P9" s="31"/>
-      <c r="Q9" s="31"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
       <c r="R9" s="17"/>
       <c r="S9" s="17"/>
       <c r="T9" s="17"/>
@@ -1026,21 +1026,21 @@
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="32"/>
-      <c r="J10" s="31"/>
-      <c r="K10" s="31"/>
-      <c r="L10" s="32"/>
-      <c r="M10" s="31"/>
-      <c r="N10" s="31"/>
-      <c r="O10" s="32"/>
-      <c r="P10" s="31"/>
-      <c r="Q10" s="31"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="18"/>
+      <c r="Q10" s="18"/>
       <c r="R10" s="17"/>
       <c r="S10" s="17"/>
       <c r="T10" s="17"/>
@@ -1048,21 +1048,21 @@
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
-      <c r="C11" s="32"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="31"/>
-      <c r="L11" s="32"/>
-      <c r="M11" s="31"/>
-      <c r="N11" s="31"/>
-      <c r="O11" s="32"/>
-      <c r="P11" s="31"/>
-      <c r="Q11" s="31"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="18"/>
+      <c r="N11" s="18"/>
+      <c r="O11" s="19"/>
+      <c r="P11" s="18"/>
+      <c r="Q11" s="18"/>
       <c r="R11" s="17"/>
       <c r="S11" s="17"/>
       <c r="T11" s="17"/>
@@ -1070,21 +1070,21 @@
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="31"/>
-      <c r="E12" s="31"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="31"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="31"/>
-      <c r="K12" s="31"/>
-      <c r="L12" s="32"/>
-      <c r="M12" s="31"/>
-      <c r="N12" s="31"/>
-      <c r="O12" s="32"/>
-      <c r="P12" s="31"/>
-      <c r="Q12" s="31"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="18"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="18"/>
+      <c r="Q12" s="18"/>
       <c r="R12" s="17"/>
       <c r="S12" s="17"/>
       <c r="T12" s="17"/>
@@ -1092,21 +1092,21 @@
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="17"/>
       <c r="B13" s="17"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="31"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="31"/>
-      <c r="L13" s="32"/>
-      <c r="M13" s="31"/>
-      <c r="N13" s="31"/>
-      <c r="O13" s="32"/>
-      <c r="P13" s="31"/>
-      <c r="Q13" s="31"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="18"/>
+      <c r="N13" s="18"/>
+      <c r="O13" s="19"/>
+      <c r="P13" s="18"/>
+      <c r="Q13" s="18"/>
       <c r="R13" s="17"/>
       <c r="S13" s="17"/>
       <c r="T13" s="17"/>
@@ -1114,21 +1114,21 @@
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="17"/>
       <c r="B14" s="17"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
-      <c r="I14" s="32"/>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="32"/>
-      <c r="M14" s="31"/>
-      <c r="N14" s="31"/>
-      <c r="O14" s="32"/>
-      <c r="P14" s="31"/>
-      <c r="Q14" s="31"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="18"/>
+      <c r="N14" s="18"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="18"/>
+      <c r="Q14" s="18"/>
       <c r="R14" s="17"/>
       <c r="S14" s="17"/>
       <c r="T14" s="17"/>
@@ -1136,21 +1136,21 @@
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="17"/>
       <c r="B15" s="17"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="31"/>
-      <c r="I15" s="32"/>
-      <c r="J15" s="31"/>
-      <c r="K15" s="31"/>
-      <c r="L15" s="32"/>
-      <c r="M15" s="31"/>
-      <c r="N15" s="31"/>
-      <c r="O15" s="32"/>
-      <c r="P15" s="31"/>
-      <c r="Q15" s="31"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="19"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="19"/>
+      <c r="M15" s="18"/>
+      <c r="N15" s="18"/>
+      <c r="O15" s="19"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
       <c r="R15" s="17"/>
       <c r="S15" s="17"/>
       <c r="T15" s="17"/>
@@ -1158,21 +1158,21 @@
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="17"/>
       <c r="B16" s="17"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="31"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="31"/>
-      <c r="K16" s="31"/>
-      <c r="L16" s="32"/>
-      <c r="M16" s="31"/>
-      <c r="N16" s="31"/>
-      <c r="O16" s="32"/>
-      <c r="P16" s="31"/>
-      <c r="Q16" s="31"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="18"/>
+      <c r="N16" s="18"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="18"/>
+      <c r="Q16" s="18"/>
       <c r="R16" s="17"/>
       <c r="S16" s="17"/>
       <c r="T16" s="17"/>
@@ -1180,21 +1180,21 @@
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="17"/>
       <c r="B17" s="17"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="31"/>
-      <c r="I17" s="32"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="31"/>
-      <c r="L17" s="32"/>
-      <c r="M17" s="31"/>
-      <c r="N17" s="31"/>
-      <c r="O17" s="32"/>
-      <c r="P17" s="31"/>
-      <c r="Q17" s="31"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="18"/>
+      <c r="N17" s="18"/>
+      <c r="O17" s="19"/>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="18"/>
       <c r="R17" s="17"/>
       <c r="S17" s="17"/>
       <c r="T17" s="17"/>
@@ -1202,21 +1202,21 @@
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="17"/>
       <c r="B18" s="17"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="31"/>
-      <c r="I18" s="32"/>
-      <c r="J18" s="31"/>
-      <c r="K18" s="31"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="31"/>
-      <c r="N18" s="31"/>
-      <c r="O18" s="32"/>
-      <c r="P18" s="31"/>
-      <c r="Q18" s="31"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="19"/>
+      <c r="P18" s="18"/>
+      <c r="Q18" s="18"/>
       <c r="R18" s="17"/>
       <c r="S18" s="17"/>
       <c r="T18" s="17"/>
@@ -1224,21 +1224,21 @@
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="17"/>
       <c r="B19" s="17"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="31"/>
-      <c r="I19" s="32"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="31"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="31"/>
-      <c r="N19" s="31"/>
-      <c r="O19" s="32"/>
-      <c r="P19" s="31"/>
-      <c r="Q19" s="31"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="18"/>
+      <c r="N19" s="18"/>
+      <c r="O19" s="19"/>
+      <c r="P19" s="18"/>
+      <c r="Q19" s="18"/>
       <c r="R19" s="17"/>
       <c r="S19" s="17"/>
       <c r="T19" s="17"/>
@@ -1246,21 +1246,21 @@
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="17"/>
       <c r="B20" s="17"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="32"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="32"/>
-      <c r="M20" s="31"/>
-      <c r="N20" s="31"/>
-      <c r="O20" s="32"/>
-      <c r="P20" s="31"/>
-      <c r="Q20" s="31"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="18"/>
+      <c r="N20" s="18"/>
+      <c r="O20" s="19"/>
+      <c r="P20" s="18"/>
+      <c r="Q20" s="18"/>
       <c r="R20" s="17"/>
       <c r="S20" s="17"/>
       <c r="T20" s="17"/>
@@ -1268,21 +1268,21 @@
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="17"/>
       <c r="B21" s="17"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="31"/>
-      <c r="H21" s="31"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="31"/>
-      <c r="K21" s="31"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="31"/>
-      <c r="N21" s="31"/>
-      <c r="O21" s="32"/>
-      <c r="P21" s="31"/>
-      <c r="Q21" s="31"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18"/>
+      <c r="L21" s="19"/>
+      <c r="M21" s="18"/>
+      <c r="N21" s="18"/>
+      <c r="O21" s="19"/>
+      <c r="P21" s="18"/>
+      <c r="Q21" s="18"/>
       <c r="R21" s="17"/>
       <c r="S21" s="17"/>
       <c r="T21" s="17"/>
@@ -1290,21 +1290,21 @@
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" s="17"/>
       <c r="B22" s="17"/>
-      <c r="C22" s="32"/>
-      <c r="D22" s="31"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="31"/>
-      <c r="H22" s="31"/>
-      <c r="I22" s="32"/>
-      <c r="J22" s="31"/>
-      <c r="K22" s="31"/>
-      <c r="L22" s="32"/>
-      <c r="M22" s="31"/>
-      <c r="N22" s="31"/>
-      <c r="O22" s="32"/>
-      <c r="P22" s="31"/>
-      <c r="Q22" s="31"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="18"/>
+      <c r="N22" s="18"/>
+      <c r="O22" s="19"/>
+      <c r="P22" s="18"/>
+      <c r="Q22" s="18"/>
       <c r="R22" s="17"/>
       <c r="S22" s="17"/>
       <c r="T22" s="17"/>
@@ -1312,21 +1312,21 @@
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" s="17"/>
       <c r="B23" s="17"/>
-      <c r="C23" s="32"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="31"/>
-      <c r="I23" s="32"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="31"/>
-      <c r="L23" s="32"/>
-      <c r="M23" s="31"/>
-      <c r="N23" s="31"/>
-      <c r="O23" s="32"/>
-      <c r="P23" s="31"/>
-      <c r="Q23" s="31"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="18"/>
+      <c r="N23" s="18"/>
+      <c r="O23" s="19"/>
+      <c r="P23" s="18"/>
+      <c r="Q23" s="18"/>
       <c r="R23" s="17"/>
       <c r="S23" s="17"/>
       <c r="T23" s="17"/>
@@ -1334,21 +1334,21 @@
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="17"/>
       <c r="B24" s="17"/>
-      <c r="C24" s="32"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="31"/>
-      <c r="H24" s="31"/>
-      <c r="I24" s="32"/>
-      <c r="J24" s="31"/>
-      <c r="K24" s="31"/>
-      <c r="L24" s="32"/>
-      <c r="M24" s="31"/>
-      <c r="N24" s="31"/>
-      <c r="O24" s="32"/>
-      <c r="P24" s="31"/>
-      <c r="Q24" s="31"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="18"/>
+      <c r="K24" s="18"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="18"/>
+      <c r="N24" s="18"/>
+      <c r="O24" s="19"/>
+      <c r="P24" s="18"/>
+      <c r="Q24" s="18"/>
       <c r="R24" s="17"/>
       <c r="S24" s="17"/>
       <c r="T24" s="17"/>
@@ -1356,21 +1356,21 @@
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="17"/>
       <c r="B25" s="17"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="31"/>
-      <c r="K25" s="31"/>
-      <c r="L25" s="32"/>
-      <c r="M25" s="31"/>
-      <c r="N25" s="31"/>
-      <c r="O25" s="32"/>
-      <c r="P25" s="31"/>
-      <c r="Q25" s="31"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="18"/>
+      <c r="N25" s="18"/>
+      <c r="O25" s="19"/>
+      <c r="P25" s="18"/>
+      <c r="Q25" s="18"/>
       <c r="R25" s="17"/>
       <c r="S25" s="17"/>
       <c r="T25" s="17"/>
@@ -1378,21 +1378,21 @@
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="17"/>
       <c r="B26" s="17"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="31"/>
-      <c r="H26" s="31"/>
-      <c r="I26" s="32"/>
-      <c r="J26" s="31"/>
-      <c r="K26" s="31"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="31"/>
-      <c r="N26" s="31"/>
-      <c r="O26" s="32"/>
-      <c r="P26" s="31"/>
-      <c r="Q26" s="31"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="18"/>
+      <c r="K26" s="18"/>
+      <c r="L26" s="19"/>
+      <c r="M26" s="18"/>
+      <c r="N26" s="18"/>
+      <c r="O26" s="19"/>
+      <c r="P26" s="18"/>
+      <c r="Q26" s="18"/>
       <c r="R26" s="17"/>
       <c r="S26" s="17"/>
       <c r="T26" s="17"/>
@@ -1400,21 +1400,21 @@
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="17"/>
       <c r="B27" s="17"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="31"/>
-      <c r="I27" s="32"/>
-      <c r="J27" s="31"/>
-      <c r="K27" s="31"/>
-      <c r="L27" s="32"/>
-      <c r="M27" s="31"/>
-      <c r="N27" s="31"/>
-      <c r="O27" s="32"/>
-      <c r="P27" s="31"/>
-      <c r="Q27" s="31"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="18"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="18"/>
+      <c r="N27" s="18"/>
+      <c r="O27" s="19"/>
+      <c r="P27" s="18"/>
+      <c r="Q27" s="18"/>
       <c r="R27" s="17"/>
       <c r="S27" s="17"/>
       <c r="T27" s="17"/>
@@ -1422,21 +1422,21 @@
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="17"/>
       <c r="B28" s="17"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="31"/>
-      <c r="I28" s="32"/>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="32"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
-      <c r="O28" s="32"/>
-      <c r="P28" s="31"/>
-      <c r="Q28" s="31"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="18"/>
+      <c r="K28" s="18"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="18"/>
+      <c r="N28" s="18"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="18"/>
+      <c r="Q28" s="18"/>
       <c r="R28" s="17"/>
       <c r="S28" s="17"/>
       <c r="T28" s="17"/>
@@ -1444,21 +1444,21 @@
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="17"/>
       <c r="B29" s="17"/>
-      <c r="C29" s="32"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="31"/>
-      <c r="I29" s="32"/>
-      <c r="J29" s="31"/>
-      <c r="K29" s="31"/>
-      <c r="L29" s="32"/>
-      <c r="M29" s="31"/>
-      <c r="N29" s="31"/>
-      <c r="O29" s="32"/>
-      <c r="P29" s="31"/>
-      <c r="Q29" s="31"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="18"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="18"/>
+      <c r="N29" s="18"/>
+      <c r="O29" s="19"/>
+      <c r="P29" s="18"/>
+      <c r="Q29" s="18"/>
       <c r="R29" s="17"/>
       <c r="S29" s="17"/>
       <c r="T29" s="17"/>
@@ -1466,21 +1466,21 @@
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" s="17"/>
       <c r="B30" s="17"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="31"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="31"/>
-      <c r="H30" s="31"/>
-      <c r="I30" s="32"/>
-      <c r="J30" s="31"/>
-      <c r="K30" s="31"/>
-      <c r="L30" s="32"/>
-      <c r="M30" s="31"/>
-      <c r="N30" s="31"/>
-      <c r="O30" s="32"/>
-      <c r="P30" s="31"/>
-      <c r="Q30" s="31"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="19"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="18"/>
+      <c r="L30" s="19"/>
+      <c r="M30" s="18"/>
+      <c r="N30" s="18"/>
+      <c r="O30" s="19"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
       <c r="R30" s="17"/>
       <c r="S30" s="17"/>
       <c r="T30" s="17"/>
@@ -1488,21 +1488,21 @@
     <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" s="17"/>
       <c r="B31" s="17"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="32"/>
-      <c r="J31" s="31"/>
-      <c r="K31" s="31"/>
-      <c r="L31" s="32"/>
-      <c r="M31" s="31"/>
-      <c r="N31" s="31"/>
-      <c r="O31" s="32"/>
-      <c r="P31" s="31"/>
-      <c r="Q31" s="31"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="18"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="18"/>
+      <c r="N31" s="18"/>
+      <c r="O31" s="19"/>
+      <c r="P31" s="18"/>
+      <c r="Q31" s="18"/>
       <c r="R31" s="17"/>
       <c r="S31" s="17"/>
       <c r="T31" s="17"/>
@@ -1510,21 +1510,21 @@
     <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" s="17"/>
       <c r="B32" s="17"/>
-      <c r="C32" s="32"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="31"/>
-      <c r="I32" s="32"/>
-      <c r="J32" s="31"/>
-      <c r="K32" s="31"/>
-      <c r="L32" s="32"/>
-      <c r="M32" s="31"/>
-      <c r="N32" s="31"/>
-      <c r="O32" s="32"/>
-      <c r="P32" s="31"/>
-      <c r="Q32" s="31"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="18"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="18"/>
+      <c r="N32" s="18"/>
+      <c r="O32" s="19"/>
+      <c r="P32" s="18"/>
+      <c r="Q32" s="18"/>
       <c r="R32" s="17"/>
       <c r="S32" s="17"/>
       <c r="T32" s="17"/>
@@ -1532,21 +1532,21 @@
     <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" s="17"/>
       <c r="B33" s="17"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="31"/>
-      <c r="E33" s="31"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="31"/>
-      <c r="H33" s="31"/>
-      <c r="I33" s="32"/>
-      <c r="J33" s="31"/>
-      <c r="K33" s="31"/>
-      <c r="L33" s="32"/>
-      <c r="M33" s="31"/>
-      <c r="N33" s="31"/>
-      <c r="O33" s="32"/>
-      <c r="P33" s="31"/>
-      <c r="Q33" s="31"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="19"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="18"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="18"/>
+      <c r="N33" s="18"/>
+      <c r="O33" s="19"/>
+      <c r="P33" s="18"/>
+      <c r="Q33" s="18"/>
       <c r="R33" s="17"/>
       <c r="S33" s="17"/>
       <c r="T33" s="17"/>
@@ -1554,21 +1554,21 @@
     <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" s="17"/>
       <c r="B34" s="17"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="31"/>
-      <c r="H34" s="31"/>
-      <c r="I34" s="32"/>
-      <c r="J34" s="31"/>
-      <c r="K34" s="31"/>
-      <c r="L34" s="32"/>
-      <c r="M34" s="31"/>
-      <c r="N34" s="31"/>
-      <c r="O34" s="32"/>
-      <c r="P34" s="31"/>
-      <c r="Q34" s="31"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="19"/>
+      <c r="J34" s="18"/>
+      <c r="K34" s="18"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="18"/>
+      <c r="N34" s="18"/>
+      <c r="O34" s="19"/>
+      <c r="P34" s="18"/>
+      <c r="Q34" s="18"/>
       <c r="R34" s="17"/>
       <c r="S34" s="17"/>
       <c r="T34" s="17"/>
@@ -1576,21 +1576,21 @@
     <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" s="17"/>
       <c r="B35" s="17"/>
-      <c r="C35" s="32"/>
-      <c r="D35" s="31"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="31"/>
-      <c r="H35" s="31"/>
-      <c r="I35" s="32"/>
-      <c r="J35" s="31"/>
-      <c r="K35" s="31"/>
-      <c r="L35" s="32"/>
-      <c r="M35" s="31"/>
-      <c r="N35" s="31"/>
-      <c r="O35" s="32"/>
-      <c r="P35" s="31"/>
-      <c r="Q35" s="31"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="19"/>
+      <c r="J35" s="18"/>
+      <c r="K35" s="18"/>
+      <c r="L35" s="19"/>
+      <c r="M35" s="18"/>
+      <c r="N35" s="18"/>
+      <c r="O35" s="19"/>
+      <c r="P35" s="18"/>
+      <c r="Q35" s="18"/>
       <c r="R35" s="17"/>
       <c r="S35" s="17"/>
       <c r="T35" s="17"/>
@@ -1598,21 +1598,21 @@
     <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" s="17"/>
       <c r="B36" s="17"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="31"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="32"/>
-      <c r="J36" s="31"/>
-      <c r="K36" s="31"/>
-      <c r="L36" s="32"/>
-      <c r="M36" s="31"/>
-      <c r="N36" s="31"/>
-      <c r="O36" s="32"/>
-      <c r="P36" s="31"/>
-      <c r="Q36" s="31"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="19"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="19"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="18"/>
+      <c r="L36" s="19"/>
+      <c r="M36" s="18"/>
+      <c r="N36" s="18"/>
+      <c r="O36" s="19"/>
+      <c r="P36" s="18"/>
+      <c r="Q36" s="18"/>
       <c r="R36" s="17"/>
       <c r="S36" s="17"/>
       <c r="T36" s="17"/>
@@ -1620,21 +1620,21 @@
     <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" s="17"/>
       <c r="B37" s="17"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="31"/>
-      <c r="H37" s="31"/>
-      <c r="I37" s="32"/>
-      <c r="J37" s="31"/>
-      <c r="K37" s="31"/>
-      <c r="L37" s="32"/>
-      <c r="M37" s="31"/>
-      <c r="N37" s="31"/>
-      <c r="O37" s="32"/>
-      <c r="P37" s="31"/>
-      <c r="Q37" s="31"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="19"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="19"/>
+      <c r="J37" s="18"/>
+      <c r="K37" s="18"/>
+      <c r="L37" s="19"/>
+      <c r="M37" s="18"/>
+      <c r="N37" s="18"/>
+      <c r="O37" s="19"/>
+      <c r="P37" s="18"/>
+      <c r="Q37" s="18"/>
       <c r="R37" s="17"/>
       <c r="S37" s="17"/>
       <c r="T37" s="17"/>
@@ -1642,21 +1642,21 @@
     <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" s="17"/>
       <c r="B38" s="17"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="31"/>
-      <c r="E38" s="31"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="31"/>
-      <c r="H38" s="31"/>
-      <c r="I38" s="32"/>
-      <c r="J38" s="31"/>
-      <c r="K38" s="31"/>
-      <c r="L38" s="32"/>
-      <c r="M38" s="31"/>
-      <c r="N38" s="31"/>
-      <c r="O38" s="32"/>
-      <c r="P38" s="31"/>
-      <c r="Q38" s="31"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="19"/>
+      <c r="J38" s="18"/>
+      <c r="K38" s="18"/>
+      <c r="L38" s="19"/>
+      <c r="M38" s="18"/>
+      <c r="N38" s="18"/>
+      <c r="O38" s="19"/>
+      <c r="P38" s="18"/>
+      <c r="Q38" s="18"/>
       <c r="R38" s="17"/>
       <c r="S38" s="17"/>
       <c r="T38" s="17"/>
@@ -1664,21 +1664,21 @@
     <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" s="17"/>
       <c r="B39" s="17"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="31"/>
-      <c r="E39" s="31"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="31"/>
-      <c r="H39" s="31"/>
-      <c r="I39" s="32"/>
-      <c r="J39" s="31"/>
-      <c r="K39" s="31"/>
-      <c r="L39" s="32"/>
-      <c r="M39" s="31"/>
-      <c r="N39" s="31"/>
-      <c r="O39" s="32"/>
-      <c r="P39" s="31"/>
-      <c r="Q39" s="31"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="19"/>
+      <c r="J39" s="18"/>
+      <c r="K39" s="18"/>
+      <c r="L39" s="19"/>
+      <c r="M39" s="18"/>
+      <c r="N39" s="18"/>
+      <c r="O39" s="19"/>
+      <c r="P39" s="18"/>
+      <c r="Q39" s="18"/>
       <c r="R39" s="17"/>
       <c r="S39" s="17"/>
       <c r="T39" s="17"/>
@@ -1686,21 +1686,21 @@
     <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" s="17"/>
       <c r="B40" s="17"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="31"/>
-      <c r="E40" s="31"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="31"/>
-      <c r="H40" s="31"/>
-      <c r="I40" s="32"/>
-      <c r="J40" s="31"/>
-      <c r="K40" s="31"/>
-      <c r="L40" s="32"/>
-      <c r="M40" s="31"/>
-      <c r="N40" s="31"/>
-      <c r="O40" s="32"/>
-      <c r="P40" s="31"/>
-      <c r="Q40" s="31"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="18"/>
+      <c r="K40" s="18"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="18"/>
+      <c r="N40" s="18"/>
+      <c r="O40" s="19"/>
+      <c r="P40" s="18"/>
+      <c r="Q40" s="18"/>
       <c r="R40" s="17"/>
       <c r="S40" s="17"/>
       <c r="T40" s="17"/>
@@ -1708,21 +1708,21 @@
     <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" s="17"/>
       <c r="B41" s="17"/>
-      <c r="C41" s="32"/>
-      <c r="D41" s="31"/>
-      <c r="E41" s="31"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="31"/>
-      <c r="I41" s="32"/>
-      <c r="J41" s="31"/>
-      <c r="K41" s="31"/>
-      <c r="L41" s="32"/>
-      <c r="M41" s="31"/>
-      <c r="N41" s="31"/>
-      <c r="O41" s="32"/>
-      <c r="P41" s="31"/>
-      <c r="Q41" s="31"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="18"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="18"/>
+      <c r="K41" s="18"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="18"/>
+      <c r="N41" s="18"/>
+      <c r="O41" s="19"/>
+      <c r="P41" s="18"/>
+      <c r="Q41" s="18"/>
       <c r="R41" s="17"/>
       <c r="S41" s="17"/>
       <c r="T41" s="17"/>
@@ -1730,21 +1730,21 @@
     <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" s="17"/>
       <c r="B42" s="17"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="31"/>
-      <c r="E42" s="31"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="31"/>
-      <c r="H42" s="31"/>
-      <c r="I42" s="32"/>
-      <c r="J42" s="31"/>
-      <c r="K42" s="31"/>
-      <c r="L42" s="32"/>
-      <c r="M42" s="31"/>
-      <c r="N42" s="31"/>
-      <c r="O42" s="32"/>
-      <c r="P42" s="31"/>
-      <c r="Q42" s="31"/>
+      <c r="C42" s="19"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="19"/>
+      <c r="G42" s="18"/>
+      <c r="H42" s="18"/>
+      <c r="I42" s="19"/>
+      <c r="J42" s="18"/>
+      <c r="K42" s="18"/>
+      <c r="L42" s="19"/>
+      <c r="M42" s="18"/>
+      <c r="N42" s="18"/>
+      <c r="O42" s="19"/>
+      <c r="P42" s="18"/>
+      <c r="Q42" s="18"/>
       <c r="R42" s="17"/>
       <c r="S42" s="17"/>
       <c r="T42" s="17"/>
@@ -1752,21 +1752,21 @@
     <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" s="17"/>
       <c r="B43" s="17"/>
-      <c r="C43" s="32"/>
-      <c r="D43" s="31"/>
-      <c r="E43" s="31"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="31"/>
-      <c r="H43" s="31"/>
-      <c r="I43" s="32"/>
-      <c r="J43" s="31"/>
-      <c r="K43" s="31"/>
-      <c r="L43" s="32"/>
-      <c r="M43" s="31"/>
-      <c r="N43" s="31"/>
-      <c r="O43" s="32"/>
-      <c r="P43" s="31"/>
-      <c r="Q43" s="31"/>
+      <c r="C43" s="19"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="19"/>
+      <c r="G43" s="18"/>
+      <c r="H43" s="18"/>
+      <c r="I43" s="19"/>
+      <c r="J43" s="18"/>
+      <c r="K43" s="18"/>
+      <c r="L43" s="19"/>
+      <c r="M43" s="18"/>
+      <c r="N43" s="18"/>
+      <c r="O43" s="19"/>
+      <c r="P43" s="18"/>
+      <c r="Q43" s="18"/>
       <c r="R43" s="17"/>
       <c r="S43" s="17"/>
       <c r="T43" s="17"/>
@@ -1774,21 +1774,21 @@
     <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" s="17"/>
       <c r="B44" s="17"/>
-      <c r="C44" s="32"/>
-      <c r="D44" s="31"/>
-      <c r="E44" s="31"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="31"/>
-      <c r="H44" s="31"/>
-      <c r="I44" s="32"/>
-      <c r="J44" s="31"/>
-      <c r="K44" s="31"/>
-      <c r="L44" s="32"/>
-      <c r="M44" s="31"/>
-      <c r="N44" s="31"/>
-      <c r="O44" s="32"/>
-      <c r="P44" s="31"/>
-      <c r="Q44" s="31"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="19"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+      <c r="I44" s="19"/>
+      <c r="J44" s="18"/>
+      <c r="K44" s="18"/>
+      <c r="L44" s="19"/>
+      <c r="M44" s="18"/>
+      <c r="N44" s="18"/>
+      <c r="O44" s="19"/>
+      <c r="P44" s="18"/>
+      <c r="Q44" s="18"/>
       <c r="R44" s="17"/>
       <c r="S44" s="17"/>
       <c r="T44" s="17"/>
@@ -1796,21 +1796,21 @@
     <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" s="17"/>
       <c r="B45" s="17"/>
-      <c r="C45" s="32"/>
-      <c r="D45" s="31"/>
-      <c r="E45" s="31"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="31"/>
-      <c r="H45" s="31"/>
-      <c r="I45" s="32"/>
-      <c r="J45" s="31"/>
-      <c r="K45" s="31"/>
-      <c r="L45" s="32"/>
-      <c r="M45" s="31"/>
-      <c r="N45" s="31"/>
-      <c r="O45" s="32"/>
-      <c r="P45" s="31"/>
-      <c r="Q45" s="31"/>
+      <c r="C45" s="19"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="19"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="19"/>
+      <c r="J45" s="18"/>
+      <c r="K45" s="18"/>
+      <c r="L45" s="19"/>
+      <c r="M45" s="18"/>
+      <c r="N45" s="18"/>
+      <c r="O45" s="19"/>
+      <c r="P45" s="18"/>
+      <c r="Q45" s="18"/>
       <c r="R45" s="17"/>
       <c r="S45" s="17"/>
       <c r="T45" s="17"/>
@@ -1818,21 +1818,21 @@
     <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" s="17"/>
       <c r="B46" s="17"/>
-      <c r="C46" s="32"/>
-      <c r="D46" s="31"/>
-      <c r="E46" s="31"/>
-      <c r="F46" s="32"/>
-      <c r="G46" s="31"/>
-      <c r="H46" s="31"/>
-      <c r="I46" s="32"/>
-      <c r="J46" s="31"/>
-      <c r="K46" s="31"/>
-      <c r="L46" s="32"/>
-      <c r="M46" s="31"/>
-      <c r="N46" s="31"/>
-      <c r="O46" s="32"/>
-      <c r="P46" s="31"/>
-      <c r="Q46" s="31"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="19"/>
+      <c r="G46" s="18"/>
+      <c r="H46" s="18"/>
+      <c r="I46" s="19"/>
+      <c r="J46" s="18"/>
+      <c r="K46" s="18"/>
+      <c r="L46" s="19"/>
+      <c r="M46" s="18"/>
+      <c r="N46" s="18"/>
+      <c r="O46" s="19"/>
+      <c r="P46" s="18"/>
+      <c r="Q46" s="18"/>
       <c r="R46" s="17"/>
       <c r="S46" s="17"/>
       <c r="T46" s="17"/>
@@ -1840,21 +1840,21 @@
     <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" s="17"/>
       <c r="B47" s="17"/>
-      <c r="C47" s="32"/>
-      <c r="D47" s="31"/>
-      <c r="E47" s="31"/>
-      <c r="F47" s="32"/>
-      <c r="G47" s="31"/>
-      <c r="H47" s="31"/>
-      <c r="I47" s="32"/>
-      <c r="J47" s="31"/>
-      <c r="K47" s="31"/>
-      <c r="L47" s="32"/>
-      <c r="M47" s="31"/>
-      <c r="N47" s="31"/>
-      <c r="O47" s="32"/>
-      <c r="P47" s="31"/>
-      <c r="Q47" s="31"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="19"/>
+      <c r="G47" s="18"/>
+      <c r="H47" s="18"/>
+      <c r="I47" s="19"/>
+      <c r="J47" s="18"/>
+      <c r="K47" s="18"/>
+      <c r="L47" s="19"/>
+      <c r="M47" s="18"/>
+      <c r="N47" s="18"/>
+      <c r="O47" s="19"/>
+      <c r="P47" s="18"/>
+      <c r="Q47" s="18"/>
       <c r="R47" s="17"/>
       <c r="S47" s="17"/>
       <c r="T47" s="17"/>
@@ -1862,21 +1862,21 @@
     <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" s="17"/>
       <c r="B48" s="17"/>
-      <c r="C48" s="32"/>
-      <c r="D48" s="31"/>
-      <c r="E48" s="31"/>
-      <c r="F48" s="32"/>
-      <c r="G48" s="31"/>
-      <c r="H48" s="31"/>
-      <c r="I48" s="32"/>
-      <c r="J48" s="31"/>
-      <c r="K48" s="31"/>
-      <c r="L48" s="32"/>
-      <c r="M48" s="31"/>
-      <c r="N48" s="31"/>
-      <c r="O48" s="32"/>
-      <c r="P48" s="31"/>
-      <c r="Q48" s="31"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="19"/>
+      <c r="G48" s="18"/>
+      <c r="H48" s="18"/>
+      <c r="I48" s="19"/>
+      <c r="J48" s="18"/>
+      <c r="K48" s="18"/>
+      <c r="L48" s="19"/>
+      <c r="M48" s="18"/>
+      <c r="N48" s="18"/>
+      <c r="O48" s="19"/>
+      <c r="P48" s="18"/>
+      <c r="Q48" s="18"/>
       <c r="R48" s="17"/>
       <c r="S48" s="17"/>
       <c r="T48" s="17"/>
@@ -1884,21 +1884,21 @@
     <row r="49" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A49" s="17"/>
       <c r="B49" s="17"/>
-      <c r="C49" s="32"/>
-      <c r="D49" s="31"/>
-      <c r="E49" s="31"/>
-      <c r="F49" s="32"/>
-      <c r="G49" s="31"/>
-      <c r="H49" s="31"/>
-      <c r="I49" s="32"/>
-      <c r="J49" s="31"/>
-      <c r="K49" s="31"/>
-      <c r="L49" s="32"/>
-      <c r="M49" s="31"/>
-      <c r="N49" s="31"/>
-      <c r="O49" s="32"/>
-      <c r="P49" s="31"/>
-      <c r="Q49" s="31"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="19"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
+      <c r="I49" s="19"/>
+      <c r="J49" s="18"/>
+      <c r="K49" s="18"/>
+      <c r="L49" s="19"/>
+      <c r="M49" s="18"/>
+      <c r="N49" s="18"/>
+      <c r="O49" s="19"/>
+      <c r="P49" s="18"/>
+      <c r="Q49" s="18"/>
       <c r="R49" s="17"/>
       <c r="S49" s="17"/>
       <c r="T49" s="17"/>
@@ -1906,21 +1906,21 @@
     <row r="50" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A50" s="17"/>
       <c r="B50" s="17"/>
-      <c r="C50" s="32"/>
-      <c r="D50" s="31"/>
-      <c r="E50" s="31"/>
-      <c r="F50" s="32"/>
-      <c r="G50" s="31"/>
-      <c r="H50" s="31"/>
-      <c r="I50" s="32"/>
-      <c r="J50" s="31"/>
-      <c r="K50" s="31"/>
-      <c r="L50" s="32"/>
-      <c r="M50" s="31"/>
-      <c r="N50" s="31"/>
-      <c r="O50" s="32"/>
-      <c r="P50" s="31"/>
-      <c r="Q50" s="31"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="19"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+      <c r="I50" s="19"/>
+      <c r="J50" s="18"/>
+      <c r="K50" s="18"/>
+      <c r="L50" s="19"/>
+      <c r="M50" s="18"/>
+      <c r="N50" s="18"/>
+      <c r="O50" s="19"/>
+      <c r="P50" s="18"/>
+      <c r="Q50" s="18"/>
       <c r="R50" s="17"/>
       <c r="S50" s="17"/>
       <c r="T50" s="17"/>
@@ -1928,21 +1928,21 @@
     <row r="51" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A51" s="17"/>
       <c r="B51" s="17"/>
-      <c r="C51" s="32"/>
-      <c r="D51" s="31"/>
-      <c r="E51" s="31"/>
-      <c r="F51" s="32"/>
-      <c r="G51" s="31"/>
-      <c r="H51" s="31"/>
-      <c r="I51" s="32"/>
-      <c r="J51" s="31"/>
-      <c r="K51" s="31"/>
-      <c r="L51" s="32"/>
-      <c r="M51" s="31"/>
-      <c r="N51" s="31"/>
-      <c r="O51" s="32"/>
-      <c r="P51" s="31"/>
-      <c r="Q51" s="31"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="18"/>
+      <c r="E51" s="18"/>
+      <c r="F51" s="19"/>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18"/>
+      <c r="I51" s="19"/>
+      <c r="J51" s="18"/>
+      <c r="K51" s="18"/>
+      <c r="L51" s="19"/>
+      <c r="M51" s="18"/>
+      <c r="N51" s="18"/>
+      <c r="O51" s="19"/>
+      <c r="P51" s="18"/>
+      <c r="Q51" s="18"/>
       <c r="R51" s="17"/>
       <c r="S51" s="17"/>
       <c r="T51" s="17"/>
@@ -1950,21 +1950,21 @@
     <row r="52" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A52" s="17"/>
       <c r="B52" s="17"/>
-      <c r="C52" s="32"/>
-      <c r="D52" s="31"/>
-      <c r="E52" s="31"/>
-      <c r="F52" s="32"/>
-      <c r="G52" s="31"/>
-      <c r="H52" s="31"/>
-      <c r="I52" s="32"/>
-      <c r="J52" s="31"/>
-      <c r="K52" s="31"/>
-      <c r="L52" s="32"/>
-      <c r="M52" s="31"/>
-      <c r="N52" s="31"/>
-      <c r="O52" s="32"/>
-      <c r="P52" s="31"/>
-      <c r="Q52" s="31"/>
+      <c r="C52" s="19"/>
+      <c r="D52" s="18"/>
+      <c r="E52" s="18"/>
+      <c r="F52" s="19"/>
+      <c r="G52" s="18"/>
+      <c r="H52" s="18"/>
+      <c r="I52" s="19"/>
+      <c r="J52" s="18"/>
+      <c r="K52" s="18"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="18"/>
+      <c r="N52" s="18"/>
+      <c r="O52" s="19"/>
+      <c r="P52" s="18"/>
+      <c r="Q52" s="18"/>
       <c r="R52" s="17"/>
       <c r="S52" s="17"/>
       <c r="T52" s="17"/>
@@ -1972,21 +1972,21 @@
     <row r="53" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A53" s="17"/>
       <c r="B53" s="17"/>
-      <c r="C53" s="32"/>
-      <c r="D53" s="31"/>
-      <c r="E53" s="31"/>
-      <c r="F53" s="32"/>
-      <c r="G53" s="31"/>
-      <c r="H53" s="31"/>
-      <c r="I53" s="32"/>
-      <c r="J53" s="31"/>
-      <c r="K53" s="31"/>
-      <c r="L53" s="32"/>
-      <c r="M53" s="31"/>
-      <c r="N53" s="31"/>
-      <c r="O53" s="32"/>
-      <c r="P53" s="31"/>
-      <c r="Q53" s="31"/>
+      <c r="C53" s="19"/>
+      <c r="D53" s="18"/>
+      <c r="E53" s="18"/>
+      <c r="F53" s="19"/>
+      <c r="G53" s="18"/>
+      <c r="H53" s="18"/>
+      <c r="I53" s="19"/>
+      <c r="J53" s="18"/>
+      <c r="K53" s="18"/>
+      <c r="L53" s="19"/>
+      <c r="M53" s="18"/>
+      <c r="N53" s="18"/>
+      <c r="O53" s="19"/>
+      <c r="P53" s="18"/>
+      <c r="Q53" s="18"/>
       <c r="R53" s="17"/>
       <c r="S53" s="17"/>
       <c r="T53" s="17"/>
@@ -1994,21 +1994,21 @@
     <row r="54" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A54" s="17"/>
       <c r="B54" s="17"/>
-      <c r="C54" s="32"/>
-      <c r="D54" s="31"/>
-      <c r="E54" s="31"/>
-      <c r="F54" s="32"/>
-      <c r="G54" s="31"/>
-      <c r="H54" s="31"/>
-      <c r="I54" s="32"/>
-      <c r="J54" s="31"/>
-      <c r="K54" s="31"/>
-      <c r="L54" s="32"/>
-      <c r="M54" s="31"/>
-      <c r="N54" s="31"/>
-      <c r="O54" s="32"/>
-      <c r="P54" s="31"/>
-      <c r="Q54" s="31"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
+      <c r="F54" s="19"/>
+      <c r="G54" s="18"/>
+      <c r="H54" s="18"/>
+      <c r="I54" s="19"/>
+      <c r="J54" s="18"/>
+      <c r="K54" s="18"/>
+      <c r="L54" s="19"/>
+      <c r="M54" s="18"/>
+      <c r="N54" s="18"/>
+      <c r="O54" s="19"/>
+      <c r="P54" s="18"/>
+      <c r="Q54" s="18"/>
       <c r="R54" s="17"/>
       <c r="S54" s="17"/>
       <c r="T54" s="17"/>
@@ -2016,21 +2016,21 @@
     <row r="55" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A55" s="17"/>
       <c r="B55" s="17"/>
-      <c r="C55" s="32"/>
-      <c r="D55" s="31"/>
-      <c r="E55" s="31"/>
-      <c r="F55" s="32"/>
-      <c r="G55" s="31"/>
-      <c r="H55" s="31"/>
-      <c r="I55" s="32"/>
-      <c r="J55" s="31"/>
-      <c r="K55" s="31"/>
-      <c r="L55" s="32"/>
-      <c r="M55" s="31"/>
-      <c r="N55" s="31"/>
-      <c r="O55" s="32"/>
-      <c r="P55" s="31"/>
-      <c r="Q55" s="31"/>
+      <c r="C55" s="19"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="19"/>
+      <c r="G55" s="18"/>
+      <c r="H55" s="18"/>
+      <c r="I55" s="19"/>
+      <c r="J55" s="18"/>
+      <c r="K55" s="18"/>
+      <c r="L55" s="19"/>
+      <c r="M55" s="18"/>
+      <c r="N55" s="18"/>
+      <c r="O55" s="19"/>
+      <c r="P55" s="18"/>
+      <c r="Q55" s="18"/>
       <c r="R55" s="17"/>
       <c r="S55" s="17"/>
       <c r="T55" s="17"/>
@@ -2038,21 +2038,21 @@
     <row r="56" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A56" s="17"/>
       <c r="B56" s="17"/>
-      <c r="C56" s="32"/>
-      <c r="D56" s="31"/>
-      <c r="E56" s="31"/>
-      <c r="F56" s="32"/>
-      <c r="G56" s="31"/>
-      <c r="H56" s="31"/>
-      <c r="I56" s="32"/>
-      <c r="J56" s="31"/>
-      <c r="K56" s="31"/>
-      <c r="L56" s="32"/>
-      <c r="M56" s="31"/>
-      <c r="N56" s="31"/>
-      <c r="O56" s="32"/>
-      <c r="P56" s="31"/>
-      <c r="Q56" s="31"/>
+      <c r="C56" s="19"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+      <c r="F56" s="19"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="18"/>
+      <c r="I56" s="19"/>
+      <c r="J56" s="18"/>
+      <c r="K56" s="18"/>
+      <c r="L56" s="19"/>
+      <c r="M56" s="18"/>
+      <c r="N56" s="18"/>
+      <c r="O56" s="19"/>
+      <c r="P56" s="18"/>
+      <c r="Q56" s="18"/>
       <c r="R56" s="17"/>
       <c r="S56" s="17"/>
       <c r="T56" s="17"/>
@@ -2060,21 +2060,21 @@
     <row r="57" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A57" s="17"/>
       <c r="B57" s="17"/>
-      <c r="C57" s="32"/>
-      <c r="D57" s="31"/>
-      <c r="E57" s="31"/>
-      <c r="F57" s="32"/>
-      <c r="G57" s="31"/>
-      <c r="H57" s="31"/>
-      <c r="I57" s="32"/>
-      <c r="J57" s="31"/>
-      <c r="K57" s="31"/>
-      <c r="L57" s="32"/>
-      <c r="M57" s="31"/>
-      <c r="N57" s="31"/>
-      <c r="O57" s="32"/>
-      <c r="P57" s="31"/>
-      <c r="Q57" s="31"/>
+      <c r="C57" s="19"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="19"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="18"/>
+      <c r="I57" s="19"/>
+      <c r="J57" s="18"/>
+      <c r="K57" s="18"/>
+      <c r="L57" s="19"/>
+      <c r="M57" s="18"/>
+      <c r="N57" s="18"/>
+      <c r="O57" s="19"/>
+      <c r="P57" s="18"/>
+      <c r="Q57" s="18"/>
       <c r="R57" s="17"/>
       <c r="S57" s="17"/>
       <c r="T57" s="17"/>
@@ -2082,21 +2082,21 @@
     <row r="58" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A58" s="17"/>
       <c r="B58" s="17"/>
-      <c r="C58" s="32"/>
-      <c r="D58" s="31"/>
-      <c r="E58" s="31"/>
-      <c r="F58" s="32"/>
-      <c r="G58" s="31"/>
-      <c r="H58" s="31"/>
-      <c r="I58" s="32"/>
-      <c r="J58" s="31"/>
-      <c r="K58" s="31"/>
-      <c r="L58" s="32"/>
-      <c r="M58" s="31"/>
-      <c r="N58" s="31"/>
-      <c r="O58" s="32"/>
-      <c r="P58" s="31"/>
-      <c r="Q58" s="31"/>
+      <c r="C58" s="19"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="18"/>
+      <c r="H58" s="18"/>
+      <c r="I58" s="19"/>
+      <c r="J58" s="18"/>
+      <c r="K58" s="18"/>
+      <c r="L58" s="19"/>
+      <c r="M58" s="18"/>
+      <c r="N58" s="18"/>
+      <c r="O58" s="19"/>
+      <c r="P58" s="18"/>
+      <c r="Q58" s="18"/>
       <c r="R58" s="17"/>
       <c r="S58" s="17"/>
       <c r="T58" s="17"/>
@@ -2104,21 +2104,21 @@
     <row r="59" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A59" s="17"/>
       <c r="B59" s="17"/>
-      <c r="C59" s="32"/>
-      <c r="D59" s="31"/>
-      <c r="E59" s="31"/>
-      <c r="F59" s="32"/>
-      <c r="G59" s="31"/>
-      <c r="H59" s="31"/>
-      <c r="I59" s="32"/>
-      <c r="J59" s="31"/>
-      <c r="K59" s="31"/>
-      <c r="L59" s="32"/>
-      <c r="M59" s="31"/>
-      <c r="N59" s="31"/>
-      <c r="O59" s="32"/>
-      <c r="P59" s="31"/>
-      <c r="Q59" s="31"/>
+      <c r="C59" s="19"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="19"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18"/>
+      <c r="I59" s="19"/>
+      <c r="J59" s="18"/>
+      <c r="K59" s="18"/>
+      <c r="L59" s="19"/>
+      <c r="M59" s="18"/>
+      <c r="N59" s="18"/>
+      <c r="O59" s="19"/>
+      <c r="P59" s="18"/>
+      <c r="Q59" s="18"/>
       <c r="R59" s="17"/>
       <c r="S59" s="17"/>
       <c r="T59" s="17"/>
@@ -2126,21 +2126,21 @@
     <row r="60" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A60" s="17"/>
       <c r="B60" s="17"/>
-      <c r="C60" s="32"/>
-      <c r="D60" s="31"/>
-      <c r="E60" s="31"/>
-      <c r="F60" s="32"/>
-      <c r="G60" s="31"/>
-      <c r="H60" s="31"/>
-      <c r="I60" s="32"/>
-      <c r="J60" s="31"/>
-      <c r="K60" s="31"/>
-      <c r="L60" s="32"/>
-      <c r="M60" s="31"/>
-      <c r="N60" s="31"/>
-      <c r="O60" s="32"/>
-      <c r="P60" s="31"/>
-      <c r="Q60" s="31"/>
+      <c r="C60" s="19"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="19"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="18"/>
+      <c r="I60" s="19"/>
+      <c r="J60" s="18"/>
+      <c r="K60" s="18"/>
+      <c r="L60" s="19"/>
+      <c r="M60" s="18"/>
+      <c r="N60" s="18"/>
+      <c r="O60" s="19"/>
+      <c r="P60" s="18"/>
+      <c r="Q60" s="18"/>
       <c r="R60" s="17"/>
       <c r="S60" s="17"/>
       <c r="T60" s="17"/>
@@ -2148,21 +2148,21 @@
     <row r="61" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A61" s="17"/>
       <c r="B61" s="17"/>
-      <c r="C61" s="32"/>
-      <c r="D61" s="31"/>
-      <c r="E61" s="31"/>
-      <c r="F61" s="32"/>
-      <c r="G61" s="31"/>
-      <c r="H61" s="31"/>
-      <c r="I61" s="32"/>
-      <c r="J61" s="31"/>
-      <c r="K61" s="31"/>
-      <c r="L61" s="32"/>
-      <c r="M61" s="31"/>
-      <c r="N61" s="31"/>
-      <c r="O61" s="32"/>
-      <c r="P61" s="31"/>
-      <c r="Q61" s="31"/>
+      <c r="C61" s="19"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+      <c r="F61" s="19"/>
+      <c r="G61" s="18"/>
+      <c r="H61" s="18"/>
+      <c r="I61" s="19"/>
+      <c r="J61" s="18"/>
+      <c r="K61" s="18"/>
+      <c r="L61" s="19"/>
+      <c r="M61" s="18"/>
+      <c r="N61" s="18"/>
+      <c r="O61" s="19"/>
+      <c r="P61" s="18"/>
+      <c r="Q61" s="18"/>
       <c r="R61" s="17"/>
       <c r="S61" s="17"/>
       <c r="T61" s="17"/>
@@ -2248,19 +2248,24 @@
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
       <c r="L64" s="12"/>
-      <c r="M64" s="18" t="s">
+      <c r="M64" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="N64" s="18"/>
-      <c r="O64" s="18"/>
-      <c r="P64" s="18"/>
-      <c r="Q64" s="18"/>
-      <c r="R64" s="18"/>
+      <c r="N64" s="32"/>
+      <c r="O64" s="32"/>
+      <c r="P64" s="32"/>
+      <c r="Q64" s="32"/>
+      <c r="R64" s="32"/>
       <c r="S64" s="1"/>
       <c r="T64" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="M64:R64"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="L3:N3"/>
+    <mergeCell ref="O3:Q3"/>
+    <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T3:T4"/>
     <mergeCell ref="A1:B1"/>
@@ -2269,11 +2274,6 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:H3"/>
-    <mergeCell ref="M64:R64"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="L3:N3"/>
-    <mergeCell ref="O3:Q3"/>
-    <mergeCell ref="R3:R4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
@@ -2281,20 +2281,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="dc189c0f-d569-423c-8bd8-1cb2ef291c21" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="dc189c0f-d569-423c-8bd8-1cb2ef291c21" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2492,14 +2492,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38AA6C2C-1214-4927-9979-113A2D4502E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52C24A3E-6A2C-40E5-B34D-1555475543C6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -2511,6 +2503,14 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38AA6C2C-1214-4927-9979-113A2D4502E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>